<commit_message>
convex combination report and clustering report updated
</commit_message>
<xml_diff>
--- a/Results/Convex_combination/Clustering/n10000/Correlation.xlsx
+++ b/Results/Convex_combination/Clustering/n10000/Correlation.xlsx
@@ -431,612 +431,612 @@
         <v>1</v>
       </c>
       <c r="B2">
-        <v>0.9903911420076684</v>
+        <v>0.9911778824120814</v>
       </c>
       <c r="C2">
-        <v>0.9851621977997472</v>
+        <v>0.9853525107839116</v>
       </c>
       <c r="D2">
-        <v>-0.6471712727828745</v>
+        <v>-0.7165456551510944</v>
       </c>
       <c r="E2">
-        <v>-0.8756990326759974</v>
+        <v>-0.8895357339952935</v>
       </c>
       <c r="F2">
-        <v>-0.8212565609126179</v>
+        <v>-0.8491672639386871</v>
       </c>
       <c r="G2">
-        <v>-0.9059584799211253</v>
+        <v>-0.9189965164729241</v>
       </c>
       <c r="H2">
-        <v>-0.7684164615882558</v>
+        <v>-0.7986974531211176</v>
       </c>
       <c r="I2">
-        <v>-0.9854888681929416</v>
+        <v>-0.9874974455209471</v>
       </c>
       <c r="J2">
-        <v>-0.3748852368878228</v>
+        <v>-0.3910163923037096</v>
       </c>
       <c r="K2">
-        <v>-0.4199817404627386</v>
+        <v>-0.4559240374918937</v>
       </c>
       <c r="L2">
-        <v>-0.4878063996884874</v>
+        <v>-0.4801667104962929</v>
       </c>
       <c r="M2">
-        <v>0.03650987127078502</v>
+        <v>-0.05355488190668174</v>
       </c>
       <c r="N2">
-        <v>0.3726634972902211</v>
+        <v>0.321264529107555</v>
       </c>
     </row>
     <row r="3">
       <c r="A3">
-        <v>0.9903911420076684</v>
+        <v>0.9911778824120814</v>
       </c>
       <c r="B3">
         <v>1</v>
       </c>
       <c r="C3">
-        <v>0.9887145488324479</v>
+        <v>0.98784402939442</v>
       </c>
       <c r="D3">
-        <v>-0.5831192290176347</v>
+        <v>-0.6651737462971744</v>
       </c>
       <c r="E3">
-        <v>-0.8682128307781293</v>
+        <v>-0.8869858503636381</v>
       </c>
       <c r="F3">
-        <v>-0.8012779699526391</v>
+        <v>-0.8363509684855724</v>
       </c>
       <c r="G3">
-        <v>-0.8839241676976729</v>
+        <v>-0.9024230642554177</v>
       </c>
       <c r="H3">
-        <v>-0.688743751833796</v>
+        <v>-0.7269781504361348</v>
       </c>
       <c r="I3">
-        <v>-0.9599446704191216</v>
+        <v>-0.9652760484795244</v>
       </c>
       <c r="J3">
-        <v>-0.4959181507907818</v>
+        <v>-0.5062520955494821</v>
       </c>
       <c r="K3">
-        <v>-0.53274235289484</v>
+        <v>-0.5609969876370733</v>
       </c>
       <c r="L3">
-        <v>-0.5957725226075659</v>
+        <v>-0.5829914252885361</v>
       </c>
       <c r="M3">
-        <v>0.02613884504472448</v>
+        <v>-0.07594196051327474</v>
       </c>
       <c r="N3">
-        <v>0.3119035040164862</v>
+        <v>0.2620976079374644</v>
       </c>
     </row>
     <row r="4">
       <c r="A4">
-        <v>0.9851621977997472</v>
+        <v>0.9853525107839116</v>
       </c>
       <c r="B4">
-        <v>0.9887145488324479</v>
+        <v>0.98784402939442</v>
       </c>
       <c r="C4">
         <v>1</v>
       </c>
       <c r="D4">
-        <v>-0.5108129214172825</v>
+        <v>-0.5903759258294538</v>
       </c>
       <c r="E4">
-        <v>-0.7945571303761106</v>
+        <v>-0.8127664917897404</v>
       </c>
       <c r="F4">
-        <v>-0.7201482414193259</v>
+        <v>-0.7554446832293878</v>
       </c>
       <c r="G4">
-        <v>-0.8244790889820389</v>
+        <v>-0.8426661935993974</v>
       </c>
       <c r="H4">
-        <v>-0.657626903740963</v>
+        <v>-0.6971048989546283</v>
       </c>
       <c r="I4">
-        <v>-0.9421825470800861</v>
+        <v>-0.9466242275876784</v>
       </c>
       <c r="J4">
-        <v>-0.44229479225444</v>
+        <v>-0.4539740435986919</v>
       </c>
       <c r="K4">
-        <v>-0.5170924147652759</v>
+        <v>-0.5459939184232456</v>
       </c>
       <c r="L4">
-        <v>-0.5652416176702975</v>
+        <v>-0.5653274358657577</v>
       </c>
       <c r="M4">
-        <v>0.10288921834841</v>
+        <v>0.0154947738248316</v>
       </c>
       <c r="N4">
-        <v>0.3755661059691884</v>
+        <v>0.3343660105024465</v>
       </c>
     </row>
     <row r="5">
       <c r="A5">
-        <v>-0.6471712727828745</v>
+        <v>-0.7165456551510944</v>
       </c>
       <c r="B5">
-        <v>-0.5831192290176347</v>
+        <v>-0.6651737462971744</v>
       </c>
       <c r="C5">
-        <v>-0.5108129214172825</v>
+        <v>-0.5903759258294538</v>
       </c>
       <c r="D5">
         <v>1</v>
       </c>
       <c r="E5">
-        <v>0.8630212107632105</v>
+        <v>0.8943927656203842</v>
       </c>
       <c r="F5">
-        <v>0.9164073560453335</v>
+        <v>0.934363973271947</v>
       </c>
       <c r="G5">
-        <v>0.8792231401723271</v>
+        <v>0.9097569187251136</v>
       </c>
       <c r="H5">
-        <v>0.9270687936904982</v>
+        <v>0.9326037420454337</v>
       </c>
       <c r="I5">
-        <v>0.7612822118580481</v>
+        <v>0.8123445620784163</v>
       </c>
       <c r="J5">
-        <v>-0.07491089996721277</v>
+        <v>0.02733490157081333</v>
       </c>
       <c r="K5">
-        <v>-0.2021396904594242</v>
+        <v>-0.07020229622526682</v>
       </c>
       <c r="L5">
-        <v>-0.07629580026058583</v>
+        <v>-0.03456087825313861</v>
       </c>
       <c r="M5">
-        <v>0.3704000393643178</v>
+        <v>0.3967240423226056</v>
       </c>
       <c r="N5">
-        <v>-0.1761085753666602</v>
+        <v>-0.1233928612101533</v>
       </c>
     </row>
     <row r="6">
       <c r="A6">
-        <v>-0.8756990326759974</v>
+        <v>-0.8895357339952935</v>
       </c>
       <c r="B6">
-        <v>-0.8682128307781293</v>
+        <v>-0.8869858503636381</v>
       </c>
       <c r="C6">
-        <v>-0.7945571303761106</v>
+        <v>-0.8127664917897404</v>
       </c>
       <c r="D6">
-        <v>0.8630212107632105</v>
+        <v>0.8943927656203842</v>
       </c>
       <c r="E6">
         <v>1</v>
       </c>
       <c r="F6">
-        <v>0.9903492783526179</v>
+        <v>0.9930574844634061</v>
       </c>
       <c r="G6">
-        <v>0.9912472136910311</v>
+        <v>0.9916704979062878</v>
       </c>
       <c r="H6">
-        <v>0.8368513004307311</v>
+        <v>0.8406059325518557</v>
       </c>
       <c r="I6">
-        <v>0.9212776735920679</v>
+        <v>0.9285902156854917</v>
       </c>
       <c r="J6">
-        <v>0.375601312617334</v>
+        <v>0.4079144503356186</v>
       </c>
       <c r="K6">
-        <v>0.287486713686584</v>
+        <v>0.3507335143087306</v>
       </c>
       <c r="L6">
-        <v>0.4015852699595497</v>
+        <v>0.3819562221360757</v>
       </c>
       <c r="M6">
-        <v>0.2368455377489306</v>
+        <v>0.3223410833546082</v>
       </c>
       <c r="N6">
-        <v>-0.1771083141033969</v>
+        <v>-0.113636341106617</v>
       </c>
     </row>
     <row r="7">
       <c r="A7">
-        <v>-0.8212565609126179</v>
+        <v>-0.8491672639386871</v>
       </c>
       <c r="B7">
-        <v>-0.8012779699526391</v>
+        <v>-0.8363509684855724</v>
       </c>
       <c r="C7">
-        <v>-0.7201482414193259</v>
+        <v>-0.7554446832293878</v>
       </c>
       <c r="D7">
-        <v>0.9164073560453335</v>
+        <v>0.934363973271947</v>
       </c>
       <c r="E7">
-        <v>0.9903492783526179</v>
+        <v>0.9930574844634061</v>
       </c>
       <c r="F7">
         <v>1</v>
       </c>
       <c r="G7">
-        <v>0.9843883278640334</v>
+        <v>0.9873148184703455</v>
       </c>
       <c r="H7">
-        <v>0.8724908906654609</v>
+        <v>0.8702195212798973</v>
       </c>
       <c r="I7">
-        <v>0.8889028403010921</v>
+        <v>0.9057161398791127</v>
       </c>
       <c r="J7">
-        <v>0.2763346510774108</v>
+        <v>0.3224399209812935</v>
       </c>
       <c r="K7">
-        <v>0.1715847690854695</v>
+        <v>0.2520717510468757</v>
       </c>
       <c r="L7">
-        <v>0.2926141659385936</v>
+        <v>0.2848669655346509</v>
       </c>
       <c r="M7">
-        <v>0.2734410288456295</v>
+        <v>0.3468174831281174</v>
       </c>
       <c r="N7">
-        <v>-0.1557770112951243</v>
+        <v>-0.09498813684352383</v>
       </c>
     </row>
     <row r="8">
       <c r="A8">
-        <v>-0.9059584799211253</v>
+        <v>-0.9189965164729241</v>
       </c>
       <c r="B8">
-        <v>-0.8839241676976729</v>
+        <v>-0.9024230642554177</v>
       </c>
       <c r="C8">
-        <v>-0.8244790889820389</v>
+        <v>-0.8426661935993974</v>
       </c>
       <c r="D8">
-        <v>0.8792231401723271</v>
+        <v>0.9097569187251136</v>
       </c>
       <c r="E8">
-        <v>0.9912472136910311</v>
+        <v>0.9916704979062878</v>
       </c>
       <c r="F8">
-        <v>0.9843883278640334</v>
+        <v>0.9873148184703455</v>
       </c>
       <c r="G8">
         <v>1</v>
       </c>
       <c r="H8">
-        <v>0.8922145056365208</v>
+        <v>0.8952620237471599</v>
       </c>
       <c r="I8">
-        <v>0.9547102998482879</v>
+        <v>0.960533854213188</v>
       </c>
       <c r="J8">
-        <v>0.2888271148789306</v>
+        <v>0.322808552959031</v>
       </c>
       <c r="K8">
-        <v>0.2312128955629236</v>
+        <v>0.2970535760890256</v>
       </c>
       <c r="L8">
-        <v>0.3429526389196763</v>
+        <v>0.3294395791684717</v>
       </c>
       <c r="M8">
-        <v>0.1691278019977862</v>
+        <v>0.2510298274403651</v>
       </c>
       <c r="N8">
-        <v>-0.2581242654714185</v>
+        <v>-0.1975451988272642</v>
       </c>
     </row>
     <row r="9">
       <c r="A9">
-        <v>-0.7684164615882558</v>
+        <v>-0.7986974531211176</v>
       </c>
       <c r="B9">
-        <v>-0.688743751833796</v>
+        <v>-0.7269781504361348</v>
       </c>
       <c r="C9">
-        <v>-0.657626903740963</v>
+        <v>-0.6971048989546283</v>
       </c>
       <c r="D9">
-        <v>0.9270687936904982</v>
+        <v>0.9326037420454337</v>
       </c>
       <c r="E9">
-        <v>0.8368513004307311</v>
+        <v>0.8406059325518557</v>
       </c>
       <c r="F9">
-        <v>0.8724908906654609</v>
+        <v>0.8702195212798973</v>
       </c>
       <c r="G9">
-        <v>0.8922145056365208</v>
+        <v>0.8952620237471599</v>
       </c>
       <c r="H9">
         <v>1</v>
       </c>
       <c r="I9">
-        <v>0.8611609016505103</v>
+        <v>0.8778584374142099</v>
       </c>
       <c r="J9">
-        <v>-0.144965869183941</v>
+        <v>-0.09657704110178822</v>
       </c>
       <c r="K9">
-        <v>-0.1576381039924295</v>
+        <v>-0.07015996173377488</v>
       </c>
       <c r="L9">
-        <v>-0.04479941455925085</v>
+        <v>-0.03315517037064933</v>
       </c>
       <c r="M9">
-        <v>0.04572354039750946</v>
+        <v>0.07885398651470703</v>
       </c>
       <c r="N9">
-        <v>-0.4388256648366168</v>
+        <v>-0.4029955615538038</v>
       </c>
     </row>
     <row r="10">
       <c r="A10">
-        <v>-0.9854888681929416</v>
+        <v>-0.9874974455209471</v>
       </c>
       <c r="B10">
-        <v>-0.9599446704191216</v>
+        <v>-0.9652760484795244</v>
       </c>
       <c r="C10">
-        <v>-0.9421825470800861</v>
+        <v>-0.9466242275876784</v>
       </c>
       <c r="D10">
-        <v>0.7612822118580481</v>
+        <v>0.8123445620784163</v>
       </c>
       <c r="E10">
-        <v>0.9212776735920679</v>
+        <v>0.9285902156854917</v>
       </c>
       <c r="F10">
-        <v>0.8889028403010921</v>
+        <v>0.9057161398791127</v>
       </c>
       <c r="G10">
-        <v>0.9547102998482879</v>
+        <v>0.960533854213188</v>
       </c>
       <c r="H10">
-        <v>0.8611609016505103</v>
+        <v>0.8778584374142099</v>
       </c>
       <c r="I10">
         <v>1</v>
       </c>
       <c r="J10">
-        <v>0.2746974916547805</v>
+        <v>0.3000352428143567</v>
       </c>
       <c r="K10">
-        <v>0.2954716828030479</v>
+        <v>0.3445295727287444</v>
       </c>
       <c r="L10">
-        <v>0.3793349582156077</v>
+        <v>0.3726463008756586</v>
       </c>
       <c r="M10">
-        <v>0.01798205829178396</v>
+        <v>0.1010314210618625</v>
       </c>
       <c r="N10">
-        <v>-0.3736114857501134</v>
+        <v>-0.3161778423934652</v>
       </c>
     </row>
     <row r="11">
       <c r="A11">
-        <v>-0.3748852368878228</v>
+        <v>-0.3910163923037096</v>
       </c>
       <c r="B11">
-        <v>-0.4959181507907818</v>
+        <v>-0.5062520955494821</v>
       </c>
       <c r="C11">
-        <v>-0.44229479225444</v>
+        <v>-0.4539740435986919</v>
       </c>
       <c r="D11">
-        <v>-0.07491089996721277</v>
+        <v>0.02733490157081333</v>
       </c>
       <c r="E11">
-        <v>0.375601312617334</v>
+        <v>0.4079144503356186</v>
       </c>
       <c r="F11">
-        <v>0.2763346510774108</v>
+        <v>0.3224399209812935</v>
       </c>
       <c r="G11">
-        <v>0.2888271148789306</v>
+        <v>0.322808552959031</v>
       </c>
       <c r="H11">
-        <v>-0.144965869183941</v>
+        <v>-0.09657704110178822</v>
       </c>
       <c r="I11">
-        <v>0.2746974916547805</v>
+        <v>0.3000352428143567</v>
       </c>
       <c r="J11">
         <v>1</v>
       </c>
       <c r="K11">
-        <v>0.9191241764500441</v>
+        <v>0.9262572760679352</v>
       </c>
       <c r="L11">
-        <v>0.9522588072614744</v>
+        <v>0.9279990345491598</v>
       </c>
       <c r="M11">
-        <v>0.09756453005562771</v>
+        <v>0.2525173785123609</v>
       </c>
       <c r="N11">
-        <v>0.2746059480503362</v>
+        <v>0.2874614839813237</v>
       </c>
     </row>
     <row r="12">
       <c r="A12">
-        <v>-0.4199817404627386</v>
+        <v>-0.4559240374918937</v>
       </c>
       <c r="B12">
-        <v>-0.53274235289484</v>
+        <v>-0.5609969876370733</v>
       </c>
       <c r="C12">
-        <v>-0.5170924147652759</v>
+        <v>-0.5459939184232456</v>
       </c>
       <c r="D12">
-        <v>-0.2021396904594242</v>
+        <v>-0.07020229622526682</v>
       </c>
       <c r="E12">
-        <v>0.287486713686584</v>
+        <v>0.3507335143087306</v>
       </c>
       <c r="F12">
-        <v>0.1715847690854695</v>
+        <v>0.2520717510468757</v>
       </c>
       <c r="G12">
-        <v>0.2312128955629236</v>
+        <v>0.2970535760890256</v>
       </c>
       <c r="H12">
-        <v>-0.1576381039924295</v>
+        <v>-0.07015996173377488</v>
       </c>
       <c r="I12">
-        <v>0.2954716828030479</v>
+        <v>0.3445295727287444</v>
       </c>
       <c r="J12">
-        <v>0.9191241764500441</v>
+        <v>0.9262572760679352</v>
       </c>
       <c r="K12">
         <v>1</v>
       </c>
       <c r="L12">
-        <v>0.9587163527965298</v>
+        <v>0.9954724219140526</v>
       </c>
       <c r="M12">
-        <v>-0.170618036556787</v>
+        <v>-0.082598144442835</v>
       </c>
       <c r="N12">
-        <v>0.05150933612200233</v>
+        <v>0.0296944366427995</v>
       </c>
     </row>
     <row r="13">
       <c r="A13">
-        <v>-0.4878063996884874</v>
+        <v>-0.4801667104962929</v>
       </c>
       <c r="B13">
-        <v>-0.5957725226075659</v>
+        <v>-0.5829914252885361</v>
       </c>
       <c r="C13">
-        <v>-0.5652416176702975</v>
+        <v>-0.5653274358657577</v>
       </c>
       <c r="D13">
-        <v>-0.07629580026058583</v>
+        <v>-0.03456087825313861</v>
       </c>
       <c r="E13">
-        <v>0.4015852699595497</v>
+        <v>0.3819562221360757</v>
       </c>
       <c r="F13">
-        <v>0.2926141659385936</v>
+        <v>0.2848669655346509</v>
       </c>
       <c r="G13">
-        <v>0.3429526389196763</v>
+        <v>0.3294395791684717</v>
       </c>
       <c r="H13">
-        <v>-0.04479941455925085</v>
+        <v>-0.03315517037064933</v>
       </c>
       <c r="I13">
-        <v>0.3793349582156077</v>
+        <v>0.3726463008756586</v>
       </c>
       <c r="J13">
-        <v>0.9522588072614744</v>
+        <v>0.9279990345491598</v>
       </c>
       <c r="K13">
-        <v>0.9587163527965298</v>
+        <v>0.9954724219140526</v>
       </c>
       <c r="L13">
         <v>1</v>
       </c>
       <c r="M13">
-        <v>-0.1552752005959236</v>
+        <v>-0.08340606998828325</v>
       </c>
       <c r="N13">
-        <v>0.0437423560618489</v>
+        <v>0.01501401793913155</v>
       </c>
     </row>
     <row r="14">
       <c r="A14">
-        <v>0.03650987127078502</v>
+        <v>-0.05355488190668174</v>
       </c>
       <c r="B14">
-        <v>0.02613884504472448</v>
+        <v>-0.07594196051327474</v>
       </c>
       <c r="C14">
-        <v>0.10288921834841</v>
+        <v>0.0154947738248316</v>
       </c>
       <c r="D14">
-        <v>0.3704000393643178</v>
+        <v>0.3967240423226056</v>
       </c>
       <c r="E14">
-        <v>0.2368455377489306</v>
+        <v>0.3223410833546082</v>
       </c>
       <c r="F14">
-        <v>0.2734410288456295</v>
+        <v>0.3468174831281174</v>
       </c>
       <c r="G14">
-        <v>0.1691278019977862</v>
+        <v>0.2510298274403651</v>
       </c>
       <c r="H14">
-        <v>0.04572354039750946</v>
+        <v>0.07885398651470703</v>
       </c>
       <c r="I14">
-        <v>0.01798205829178396</v>
+        <v>0.1010314210618625</v>
       </c>
       <c r="J14">
-        <v>0.09756453005562771</v>
+        <v>0.2525173785123609</v>
       </c>
       <c r="K14">
-        <v>-0.170618036556787</v>
+        <v>-0.082598144442835</v>
       </c>
       <c r="L14">
-        <v>-0.1552752005959236</v>
+        <v>-0.08340606998828325</v>
       </c>
       <c r="M14">
         <v>1</v>
       </c>
       <c r="N14">
-        <v>0.5643010028229847</v>
+        <v>0.6321141367226342</v>
       </c>
     </row>
     <row r="15">
       <c r="A15">
-        <v>0.3726634972902211</v>
+        <v>0.321264529107555</v>
       </c>
       <c r="B15">
-        <v>0.3119035040164862</v>
+        <v>0.2620976079374644</v>
       </c>
       <c r="C15">
-        <v>0.3755661059691884</v>
+        <v>0.3343660105024465</v>
       </c>
       <c r="D15">
-        <v>-0.1761085753666602</v>
+        <v>-0.1233928612101533</v>
       </c>
       <c r="E15">
-        <v>-0.1771083141033969</v>
+        <v>-0.113636341106617</v>
       </c>
       <c r="F15">
-        <v>-0.1557770112951243</v>
+        <v>-0.09498813684352383</v>
       </c>
       <c r="G15">
-        <v>-0.2581242654714185</v>
+        <v>-0.1975451988272642</v>
       </c>
       <c r="H15">
-        <v>-0.4388256648366168</v>
+        <v>-0.4029955615538038</v>
       </c>
       <c r="I15">
-        <v>-0.3736114857501134</v>
+        <v>-0.3161778423934652</v>
       </c>
       <c r="J15">
-        <v>0.2746059480503362</v>
+        <v>0.2874614839813237</v>
       </c>
       <c r="K15">
-        <v>0.05150933612200233</v>
+        <v>0.0296944366427995</v>
       </c>
       <c r="L15">
-        <v>0.0437423560618489</v>
+        <v>0.01501401793913155</v>
       </c>
       <c r="M15">
-        <v>0.5643010028229847</v>
+        <v>0.6321141367226342</v>
       </c>
       <c r="N15">
         <v>1</v>

</xml_diff>

<commit_message>
convex combination report updated
</commit_message>
<xml_diff>
--- a/Results/Convex_combination/Clustering/n10000/Correlation.xlsx
+++ b/Results/Convex_combination/Clustering/n10000/Correlation.xlsx
@@ -351,7 +351,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:N15"/>
+  <dimension ref="A1:M14"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" s="1" customFormat="1">
@@ -417,11 +417,6 @@
       </c>
       <c r="M1" s="1" t="inlineStr">
         <is>
-          <t>Var_H_Fisher</t>
-        </is>
-      </c>
-      <c r="N1" s="1" t="inlineStr">
-        <is>
           <t>Var_C_Shannon</t>
         </is>
       </c>
@@ -437,7 +432,7 @@
         <v>0.9853525107839116</v>
       </c>
       <c r="D2">
-        <v>-0.7165456551510944</v>
+        <v>-0.6868368075238475</v>
       </c>
       <c r="E2">
         <v>-0.8895357339952935</v>
@@ -449,7 +444,7 @@
         <v>-0.9189965164729241</v>
       </c>
       <c r="H2">
-        <v>-0.7986974531211176</v>
+        <v>-0.8508790821654865</v>
       </c>
       <c r="I2">
         <v>-0.9874974455209471</v>
@@ -464,9 +459,6 @@
         <v>-0.4801667104962929</v>
       </c>
       <c r="M2">
-        <v>-0.05355488190668174</v>
-      </c>
-      <c r="N2">
         <v>0.321264529107555</v>
       </c>
     </row>
@@ -481,7 +473,7 @@
         <v>0.98784402939442</v>
       </c>
       <c r="D3">
-        <v>-0.6651737462971744</v>
+        <v>-0.6607895329185643</v>
       </c>
       <c r="E3">
         <v>-0.8869858503636381</v>
@@ -493,7 +485,7 @@
         <v>-0.9024230642554177</v>
       </c>
       <c r="H3">
-        <v>-0.7269781504361348</v>
+        <v>-0.7931591847979717</v>
       </c>
       <c r="I3">
         <v>-0.9652760484795244</v>
@@ -508,9 +500,6 @@
         <v>-0.5829914252885361</v>
       </c>
       <c r="M3">
-        <v>-0.07594196051327474</v>
-      </c>
-      <c r="N3">
         <v>0.2620976079374644</v>
       </c>
     </row>
@@ -525,7 +514,7 @@
         <v>1</v>
       </c>
       <c r="D4">
-        <v>-0.5903759258294538</v>
+        <v>-0.5684629180817508</v>
       </c>
       <c r="E4">
         <v>-0.8127664917897404</v>
@@ -537,7 +526,7 @@
         <v>-0.8426661935993974</v>
       </c>
       <c r="H4">
-        <v>-0.6971048989546283</v>
+        <v>-0.7545446553645658</v>
       </c>
       <c r="I4">
         <v>-0.9466242275876784</v>
@@ -552,54 +541,48 @@
         <v>-0.5653274358657577</v>
       </c>
       <c r="M4">
-        <v>0.0154947738248316</v>
-      </c>
-      <c r="N4">
         <v>0.3343660105024465</v>
       </c>
     </row>
     <row r="5">
       <c r="A5">
-        <v>-0.7165456551510944</v>
+        <v>-0.6868368075238475</v>
       </c>
       <c r="B5">
-        <v>-0.6651737462971744</v>
+        <v>-0.6607895329185643</v>
       </c>
       <c r="C5">
-        <v>-0.5903759258294538</v>
+        <v>-0.5684629180817508</v>
       </c>
       <c r="D5">
         <v>1</v>
       </c>
       <c r="E5">
-        <v>0.8943927656203842</v>
+        <v>0.9039592040280597</v>
       </c>
       <c r="F5">
-        <v>0.934363973271947</v>
+        <v>0.9348953152829155</v>
       </c>
       <c r="G5">
-        <v>0.9097569187251136</v>
+        <v>0.8911933898543798</v>
       </c>
       <c r="H5">
-        <v>0.9326037420454337</v>
+        <v>0.8744589719426411</v>
       </c>
       <c r="I5">
-        <v>0.8123445620784163</v>
+        <v>0.7705413742891014</v>
       </c>
       <c r="J5">
-        <v>0.02733490157081333</v>
+        <v>0.1915930965209494</v>
       </c>
       <c r="K5">
-        <v>-0.07020229622526682</v>
+        <v>0.02623284654614912</v>
       </c>
       <c r="L5">
-        <v>-0.03456087825313861</v>
+        <v>0.05655541052515511</v>
       </c>
       <c r="M5">
-        <v>0.3967240423226056</v>
-      </c>
-      <c r="N5">
-        <v>-0.1233928612101533</v>
+        <v>0.08191201908684906</v>
       </c>
     </row>
     <row r="6">
@@ -613,7 +596,7 @@
         <v>-0.8127664917897404</v>
       </c>
       <c r="D6">
-        <v>0.8943927656203842</v>
+        <v>0.9039592040280597</v>
       </c>
       <c r="E6">
         <v>1</v>
@@ -625,7 +608,7 @@
         <v>0.9916704979062878</v>
       </c>
       <c r="H6">
-        <v>0.8406059325518557</v>
+        <v>0.9036353510935313</v>
       </c>
       <c r="I6">
         <v>0.9285902156854917</v>
@@ -640,9 +623,6 @@
         <v>0.3819562221360757</v>
       </c>
       <c r="M6">
-        <v>0.3223410833546082</v>
-      </c>
-      <c r="N6">
         <v>-0.113636341106617</v>
       </c>
     </row>
@@ -657,7 +637,7 @@
         <v>-0.7554446832293878</v>
       </c>
       <c r="D7">
-        <v>0.934363973271947</v>
+        <v>0.9348953152829155</v>
       </c>
       <c r="E7">
         <v>0.9930574844634061</v>
@@ -669,7 +649,7 @@
         <v>0.9873148184703455</v>
       </c>
       <c r="H7">
-        <v>0.8702195212798973</v>
+        <v>0.9231783488186942</v>
       </c>
       <c r="I7">
         <v>0.9057161398791127</v>
@@ -684,9 +664,6 @@
         <v>0.2848669655346509</v>
       </c>
       <c r="M7">
-        <v>0.3468174831281174</v>
-      </c>
-      <c r="N7">
         <v>-0.09498813684352383</v>
       </c>
     </row>
@@ -701,7 +678,7 @@
         <v>-0.8426661935993974</v>
       </c>
       <c r="D8">
-        <v>0.9097569187251136</v>
+        <v>0.8911933898543798</v>
       </c>
       <c r="E8">
         <v>0.9916704979062878</v>
@@ -713,7 +690,7 @@
         <v>1</v>
       </c>
       <c r="H8">
-        <v>0.8952620237471599</v>
+        <v>0.9446435007771408</v>
       </c>
       <c r="I8">
         <v>0.960533854213188</v>
@@ -728,54 +705,48 @@
         <v>0.3294395791684717</v>
       </c>
       <c r="M8">
-        <v>0.2510298274403651</v>
-      </c>
-      <c r="N8">
         <v>-0.1975451988272642</v>
       </c>
     </row>
     <row r="9">
       <c r="A9">
-        <v>-0.7986974531211176</v>
+        <v>-0.8508790821654865</v>
       </c>
       <c r="B9">
-        <v>-0.7269781504361348</v>
+        <v>-0.7931591847979717</v>
       </c>
       <c r="C9">
-        <v>-0.6971048989546283</v>
+        <v>-0.7545446553645658</v>
       </c>
       <c r="D9">
-        <v>0.9326037420454337</v>
+        <v>0.8744589719426411</v>
       </c>
       <c r="E9">
-        <v>0.8406059325518557</v>
+        <v>0.9036353510935313</v>
       </c>
       <c r="F9">
-        <v>0.8702195212798973</v>
+        <v>0.9231783488186942</v>
       </c>
       <c r="G9">
-        <v>0.8952620237471599</v>
+        <v>0.9446435007771408</v>
       </c>
       <c r="H9">
         <v>1</v>
       </c>
       <c r="I9">
-        <v>0.8778584374142099</v>
+        <v>0.9206053567149425</v>
       </c>
       <c r="J9">
-        <v>-0.09657704110178822</v>
+        <v>0.02376327216464478</v>
       </c>
       <c r="K9">
-        <v>-0.07015996173377488</v>
+        <v>0.01964597246437448</v>
       </c>
       <c r="L9">
-        <v>-0.03315517037064933</v>
+        <v>0.05532678735285265</v>
       </c>
       <c r="M9">
-        <v>0.07885398651470703</v>
-      </c>
-      <c r="N9">
-        <v>-0.4029955615538038</v>
+        <v>-0.3474678719191252</v>
       </c>
     </row>
     <row r="10">
@@ -789,7 +760,7 @@
         <v>-0.9466242275876784</v>
       </c>
       <c r="D10">
-        <v>0.8123445620784163</v>
+        <v>0.7705413742891014</v>
       </c>
       <c r="E10">
         <v>0.9285902156854917</v>
@@ -801,7 +772,7 @@
         <v>0.960533854213188</v>
       </c>
       <c r="H10">
-        <v>0.8778584374142099</v>
+        <v>0.9206053567149425</v>
       </c>
       <c r="I10">
         <v>1</v>
@@ -816,9 +787,6 @@
         <v>0.3726463008756586</v>
       </c>
       <c r="M10">
-        <v>0.1010314210618625</v>
-      </c>
-      <c r="N10">
         <v>-0.3161778423934652</v>
       </c>
     </row>
@@ -833,7 +801,7 @@
         <v>-0.4539740435986919</v>
       </c>
       <c r="D11">
-        <v>0.02733490157081333</v>
+        <v>0.1915930965209494</v>
       </c>
       <c r="E11">
         <v>0.4079144503356186</v>
@@ -845,7 +813,7 @@
         <v>0.322808552959031</v>
       </c>
       <c r="H11">
-        <v>-0.09657704110178822</v>
+        <v>0.02376327216464478</v>
       </c>
       <c r="I11">
         <v>0.3000352428143567</v>
@@ -860,9 +828,6 @@
         <v>0.9279990345491598</v>
       </c>
       <c r="M11">
-        <v>0.2525173785123609</v>
-      </c>
-      <c r="N11">
         <v>0.2874614839813237</v>
       </c>
     </row>
@@ -877,7 +842,7 @@
         <v>-0.5459939184232456</v>
       </c>
       <c r="D12">
-        <v>-0.07020229622526682</v>
+        <v>0.02623284654614912</v>
       </c>
       <c r="E12">
         <v>0.3507335143087306</v>
@@ -889,7 +854,7 @@
         <v>0.2970535760890256</v>
       </c>
       <c r="H12">
-        <v>-0.07015996173377488</v>
+        <v>0.01964597246437448</v>
       </c>
       <c r="I12">
         <v>0.3445295727287444</v>
@@ -904,9 +869,6 @@
         <v>0.9954724219140526</v>
       </c>
       <c r="M12">
-        <v>-0.082598144442835</v>
-      </c>
-      <c r="N12">
         <v>0.0296944366427995</v>
       </c>
     </row>
@@ -921,7 +883,7 @@
         <v>-0.5653274358657577</v>
       </c>
       <c r="D13">
-        <v>-0.03456087825313861</v>
+        <v>0.05655541052515511</v>
       </c>
       <c r="E13">
         <v>0.3819562221360757</v>
@@ -933,7 +895,7 @@
         <v>0.3294395791684717</v>
       </c>
       <c r="H13">
-        <v>-0.03315517037064933</v>
+        <v>0.05532678735285265</v>
       </c>
       <c r="I13">
         <v>0.3726463008756586</v>
@@ -948,97 +910,47 @@
         <v>1</v>
       </c>
       <c r="M13">
-        <v>-0.08340606998828325</v>
-      </c>
-      <c r="N13">
         <v>0.01501401793913155</v>
       </c>
     </row>
     <row r="14">
       <c r="A14">
-        <v>-0.05355488190668174</v>
+        <v>0.321264529107555</v>
       </c>
       <c r="B14">
-        <v>-0.07594196051327474</v>
+        <v>0.2620976079374644</v>
       </c>
       <c r="C14">
-        <v>0.0154947738248316</v>
+        <v>0.3343660105024465</v>
       </c>
       <c r="D14">
-        <v>0.3967240423226056</v>
+        <v>0.08191201908684906</v>
       </c>
       <c r="E14">
-        <v>0.3223410833546082</v>
+        <v>-0.113636341106617</v>
       </c>
       <c r="F14">
-        <v>0.3468174831281174</v>
+        <v>-0.09498813684352383</v>
       </c>
       <c r="G14">
-        <v>0.2510298274403651</v>
+        <v>-0.1975451988272642</v>
       </c>
       <c r="H14">
-        <v>0.07885398651470703</v>
+        <v>-0.3474678719191252</v>
       </c>
       <c r="I14">
-        <v>0.1010314210618625</v>
+        <v>-0.3161778423934652</v>
       </c>
       <c r="J14">
-        <v>0.2525173785123609</v>
+        <v>0.2874614839813237</v>
       </c>
       <c r="K14">
-        <v>-0.082598144442835</v>
+        <v>0.0296944366427995</v>
       </c>
       <c r="L14">
-        <v>-0.08340606998828325</v>
+        <v>0.01501401793913155</v>
       </c>
       <c r="M14">
-        <v>1</v>
-      </c>
-      <c r="N14">
-        <v>0.6321141367226342</v>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15">
-        <v>0.321264529107555</v>
-      </c>
-      <c r="B15">
-        <v>0.2620976079374644</v>
-      </c>
-      <c r="C15">
-        <v>0.3343660105024465</v>
-      </c>
-      <c r="D15">
-        <v>-0.1233928612101533</v>
-      </c>
-      <c r="E15">
-        <v>-0.113636341106617</v>
-      </c>
-      <c r="F15">
-        <v>-0.09498813684352383</v>
-      </c>
-      <c r="G15">
-        <v>-0.1975451988272642</v>
-      </c>
-      <c r="H15">
-        <v>-0.4029955615538038</v>
-      </c>
-      <c r="I15">
-        <v>-0.3161778423934652</v>
-      </c>
-      <c r="J15">
-        <v>0.2874614839813237</v>
-      </c>
-      <c r="K15">
-        <v>0.0296944366427995</v>
-      </c>
-      <c r="L15">
-        <v>0.01501401793913155</v>
-      </c>
-      <c r="M15">
-        <v>0.6321141367226342</v>
-      </c>
-      <c r="N15">
         <v>1</v>
       </c>
     </row>

</xml_diff>